<commit_message>
Edite Au sales Aug.2026
</commit_message>
<xml_diff>
--- a/sales_data.xlsx.xlsx
+++ b/sales_data.xlsx.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Desktop 2025+2026\2025\خطط تطوير\AI\final\تحليل شهري\Claude + GitHub\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C7B1DF2-E7E9-4F13-934A-214250A29F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D37699F-7E1B-4AB9-A2AC-DD8132B0CBE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{B1B892D3-C8DC-437F-A938-CC0527360C32}"/>
   </bookViews>
@@ -733,6 +733,21 @@
     <xf numFmtId="165" fontId="7" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="3" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="44" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -806,21 +821,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="4" fillId="10" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="3" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1149,199 +1149,199 @@
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="38" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="62" t="s">
+      <c r="C2" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="D2" s="62"/>
-      <c r="E2" s="62"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="62"/>
-      <c r="H2" s="62"/>
-      <c r="I2" s="62"/>
-      <c r="J2" s="62"/>
-      <c r="K2" s="62"/>
-      <c r="L2" s="62"/>
-      <c r="M2" s="62"/>
-      <c r="N2" s="62"/>
-      <c r="O2" s="62"/>
-      <c r="P2" s="62"/>
-      <c r="Q2" s="62"/>
-      <c r="R2" s="62"/>
-      <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="62"/>
-      <c r="W2" s="62"/>
-      <c r="X2" s="62"/>
-      <c r="Y2" s="62"/>
-      <c r="Z2" s="62"/>
-      <c r="AA2" s="62"/>
-      <c r="AB2" s="62"/>
-      <c r="AC2" s="62"/>
-      <c r="AD2" s="62"/>
-      <c r="AE2" s="62"/>
-      <c r="AF2" s="62"/>
-      <c r="AG2" s="62"/>
-      <c r="AH2" s="62"/>
-      <c r="AI2" s="62"/>
-      <c r="AJ2" s="62"/>
-      <c r="AK2" s="62"/>
-      <c r="AL2" s="62"/>
-      <c r="AM2" s="62"/>
-      <c r="AN2" s="62"/>
-      <c r="AO2" s="62"/>
-      <c r="AP2" s="62"/>
-      <c r="AQ2" s="62"/>
-      <c r="AR2" s="62"/>
-      <c r="AS2" s="62"/>
-      <c r="AT2" s="62"/>
-      <c r="AU2" s="62"/>
-      <c r="AV2" s="62"/>
-      <c r="AW2" s="62"/>
-      <c r="AX2" s="62"/>
-      <c r="AY2" s="62"/>
-      <c r="AZ2" s="62"/>
-      <c r="BA2" s="62"/>
-      <c r="BB2" s="62"/>
-      <c r="BC2" s="62"/>
-      <c r="BD2" s="62"/>
-      <c r="BE2" s="62"/>
-      <c r="BF2" s="62"/>
-      <c r="BG2" s="62"/>
-      <c r="BH2" s="62"/>
-      <c r="BI2" s="62"/>
-      <c r="BJ2" s="62"/>
-      <c r="BK2" s="62"/>
-      <c r="BL2" s="62"/>
-      <c r="BM2" s="62"/>
-      <c r="BN2" s="62"/>
-      <c r="BO2" s="62"/>
-      <c r="BP2" s="62"/>
-      <c r="BQ2" s="62"/>
-      <c r="BR2" s="62"/>
-      <c r="BS2" s="62"/>
-      <c r="BT2" s="62"/>
-      <c r="BU2" s="62"/>
-      <c r="BV2" s="62"/>
-      <c r="BW2" s="62"/>
-      <c r="BX2" s="62"/>
-      <c r="BY2" s="62"/>
-      <c r="BZ2" s="62"/>
-      <c r="CA2" s="62"/>
-      <c r="CB2" s="62"/>
-      <c r="CC2" s="62"/>
-      <c r="CD2" s="62"/>
-      <c r="CE2" s="62"/>
-      <c r="CF2" s="62"/>
-      <c r="CG2" s="62"/>
-      <c r="CH2" s="62"/>
+      <c r="D2" s="37"/>
+      <c r="E2" s="37"/>
+      <c r="F2" s="37"/>
+      <c r="G2" s="37"/>
+      <c r="H2" s="37"/>
+      <c r="I2" s="37"/>
+      <c r="J2" s="37"/>
+      <c r="K2" s="37"/>
+      <c r="L2" s="37"/>
+      <c r="M2" s="37"/>
+      <c r="N2" s="37"/>
+      <c r="O2" s="37"/>
+      <c r="P2" s="37"/>
+      <c r="Q2" s="37"/>
+      <c r="R2" s="37"/>
+      <c r="S2" s="37"/>
+      <c r="T2" s="37"/>
+      <c r="U2" s="37"/>
+      <c r="V2" s="37"/>
+      <c r="W2" s="37"/>
+      <c r="X2" s="37"/>
+      <c r="Y2" s="37"/>
+      <c r="Z2" s="37"/>
+      <c r="AA2" s="37"/>
+      <c r="AB2" s="37"/>
+      <c r="AC2" s="37"/>
+      <c r="AD2" s="37"/>
+      <c r="AE2" s="37"/>
+      <c r="AF2" s="37"/>
+      <c r="AG2" s="37"/>
+      <c r="AH2" s="37"/>
+      <c r="AI2" s="37"/>
+      <c r="AJ2" s="37"/>
+      <c r="AK2" s="37"/>
+      <c r="AL2" s="37"/>
+      <c r="AM2" s="37"/>
+      <c r="AN2" s="37"/>
+      <c r="AO2" s="37"/>
+      <c r="AP2" s="37"/>
+      <c r="AQ2" s="37"/>
+      <c r="AR2" s="37"/>
+      <c r="AS2" s="37"/>
+      <c r="AT2" s="37"/>
+      <c r="AU2" s="37"/>
+      <c r="AV2" s="37"/>
+      <c r="AW2" s="37"/>
+      <c r="AX2" s="37"/>
+      <c r="AY2" s="37"/>
+      <c r="AZ2" s="37"/>
+      <c r="BA2" s="37"/>
+      <c r="BB2" s="37"/>
+      <c r="BC2" s="37"/>
+      <c r="BD2" s="37"/>
+      <c r="BE2" s="37"/>
+      <c r="BF2" s="37"/>
+      <c r="BG2" s="37"/>
+      <c r="BH2" s="37"/>
+      <c r="BI2" s="37"/>
+      <c r="BJ2" s="37"/>
+      <c r="BK2" s="37"/>
+      <c r="BL2" s="37"/>
+      <c r="BM2" s="37"/>
+      <c r="BN2" s="37"/>
+      <c r="BO2" s="37"/>
+      <c r="BP2" s="37"/>
+      <c r="BQ2" s="37"/>
+      <c r="BR2" s="37"/>
+      <c r="BS2" s="37"/>
+      <c r="BT2" s="37"/>
+      <c r="BU2" s="37"/>
+      <c r="BV2" s="37"/>
+      <c r="BW2" s="37"/>
+      <c r="BX2" s="37"/>
+      <c r="BY2" s="37"/>
+      <c r="BZ2" s="37"/>
+      <c r="CA2" s="37"/>
+      <c r="CB2" s="37"/>
+      <c r="CC2" s="37"/>
+      <c r="CD2" s="37"/>
+      <c r="CE2" s="37"/>
+      <c r="CF2" s="37"/>
+      <c r="CG2" s="37"/>
+      <c r="CH2" s="37"/>
     </row>
     <row r="3" spans="1:86" ht="18" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B3" s="64"/>
-      <c r="C3" s="65">
+      <c r="B3" s="39"/>
+      <c r="C3" s="40">
         <v>2020</v>
       </c>
-      <c r="D3" s="65"/>
-      <c r="E3" s="65"/>
-      <c r="F3" s="65"/>
-      <c r="G3" s="65"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-      <c r="J3" s="65"/>
-      <c r="K3" s="65"/>
-      <c r="L3" s="65"/>
-      <c r="M3" s="65"/>
-      <c r="N3" s="65"/>
-      <c r="O3" s="65">
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="40">
         <v>2021</v>
       </c>
-      <c r="P3" s="65"/>
-      <c r="Q3" s="65"/>
-      <c r="R3" s="65"/>
-      <c r="S3" s="65"/>
-      <c r="T3" s="65"/>
-      <c r="U3" s="65"/>
-      <c r="V3" s="65"/>
-      <c r="W3" s="65"/>
-      <c r="X3" s="65"/>
-      <c r="Y3" s="65"/>
-      <c r="Z3" s="65"/>
-      <c r="AA3" s="61">
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="40"/>
+      <c r="S3" s="40"/>
+      <c r="T3" s="40"/>
+      <c r="U3" s="40"/>
+      <c r="V3" s="40"/>
+      <c r="W3" s="40"/>
+      <c r="X3" s="40"/>
+      <c r="Y3" s="40"/>
+      <c r="Z3" s="40"/>
+      <c r="AA3" s="36">
         <v>2022</v>
       </c>
-      <c r="AB3" s="61"/>
-      <c r="AC3" s="61"/>
-      <c r="AD3" s="61"/>
-      <c r="AE3" s="61"/>
-      <c r="AF3" s="61"/>
-      <c r="AG3" s="61"/>
-      <c r="AH3" s="61"/>
-      <c r="AI3" s="61"/>
-      <c r="AJ3" s="61"/>
-      <c r="AK3" s="61"/>
-      <c r="AL3" s="61"/>
-      <c r="AM3" s="61">
+      <c r="AB3" s="36"/>
+      <c r="AC3" s="36"/>
+      <c r="AD3" s="36"/>
+      <c r="AE3" s="36"/>
+      <c r="AF3" s="36"/>
+      <c r="AG3" s="36"/>
+      <c r="AH3" s="36"/>
+      <c r="AI3" s="36"/>
+      <c r="AJ3" s="36"/>
+      <c r="AK3" s="36"/>
+      <c r="AL3" s="36"/>
+      <c r="AM3" s="36">
         <v>2023</v>
       </c>
-      <c r="AN3" s="61"/>
-      <c r="AO3" s="61"/>
-      <c r="AP3" s="61"/>
-      <c r="AQ3" s="61"/>
-      <c r="AR3" s="61"/>
-      <c r="AS3" s="61"/>
-      <c r="AT3" s="61"/>
-      <c r="AU3" s="61"/>
-      <c r="AV3" s="61"/>
-      <c r="AW3" s="61"/>
-      <c r="AX3" s="61"/>
-      <c r="AY3" s="61">
+      <c r="AN3" s="36"/>
+      <c r="AO3" s="36"/>
+      <c r="AP3" s="36"/>
+      <c r="AQ3" s="36"/>
+      <c r="AR3" s="36"/>
+      <c r="AS3" s="36"/>
+      <c r="AT3" s="36"/>
+      <c r="AU3" s="36"/>
+      <c r="AV3" s="36"/>
+      <c r="AW3" s="36"/>
+      <c r="AX3" s="36"/>
+      <c r="AY3" s="36">
         <v>2024</v>
       </c>
-      <c r="AZ3" s="61"/>
-      <c r="BA3" s="61"/>
-      <c r="BB3" s="61"/>
-      <c r="BC3" s="61"/>
-      <c r="BD3" s="61"/>
-      <c r="BE3" s="61"/>
-      <c r="BF3" s="61"/>
-      <c r="BG3" s="61"/>
-      <c r="BH3" s="61"/>
-      <c r="BI3" s="61"/>
-      <c r="BJ3" s="61"/>
-      <c r="BK3" s="61">
+      <c r="AZ3" s="36"/>
+      <c r="BA3" s="36"/>
+      <c r="BB3" s="36"/>
+      <c r="BC3" s="36"/>
+      <c r="BD3" s="36"/>
+      <c r="BE3" s="36"/>
+      <c r="BF3" s="36"/>
+      <c r="BG3" s="36"/>
+      <c r="BH3" s="36"/>
+      <c r="BI3" s="36"/>
+      <c r="BJ3" s="36"/>
+      <c r="BK3" s="36">
         <v>2025</v>
       </c>
-      <c r="BL3" s="61"/>
-      <c r="BM3" s="61"/>
-      <c r="BN3" s="61"/>
-      <c r="BO3" s="61"/>
-      <c r="BP3" s="61"/>
-      <c r="BQ3" s="61"/>
-      <c r="BR3" s="61"/>
-      <c r="BS3" s="61"/>
-      <c r="BT3" s="61"/>
-      <c r="BU3" s="61"/>
-      <c r="BV3" s="61"/>
-      <c r="BW3" s="61">
+      <c r="BL3" s="36"/>
+      <c r="BM3" s="36"/>
+      <c r="BN3" s="36"/>
+      <c r="BO3" s="36"/>
+      <c r="BP3" s="36"/>
+      <c r="BQ3" s="36"/>
+      <c r="BR3" s="36"/>
+      <c r="BS3" s="36"/>
+      <c r="BT3" s="36"/>
+      <c r="BU3" s="36"/>
+      <c r="BV3" s="36"/>
+      <c r="BW3" s="36">
         <v>2026</v>
       </c>
-      <c r="BX3" s="61"/>
-      <c r="BY3" s="61"/>
-      <c r="BZ3" s="61"/>
-      <c r="CA3" s="61"/>
-      <c r="CB3" s="61"/>
-      <c r="CC3" s="61"/>
-      <c r="CD3" s="61"/>
-      <c r="CE3" s="61"/>
-      <c r="CF3" s="61"/>
-      <c r="CG3" s="61"/>
-      <c r="CH3" s="61"/>
+      <c r="BX3" s="36"/>
+      <c r="BY3" s="36"/>
+      <c r="BZ3" s="36"/>
+      <c r="CA3" s="36"/>
+      <c r="CB3" s="36"/>
+      <c r="CC3" s="36"/>
+      <c r="CD3" s="36"/>
+      <c r="CE3" s="36"/>
+      <c r="CF3" s="36"/>
+      <c r="CG3" s="36"/>
+      <c r="CH3" s="36"/>
     </row>
     <row r="4" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -1604,7 +1604,7 @@
       </c>
     </row>
     <row r="5" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="41" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
@@ -1864,7 +1864,7 @@
       </c>
     </row>
     <row r="6" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="37"/>
+      <c r="A6" s="42"/>
       <c r="B6" s="8" t="s">
         <v>5</v>
       </c>
@@ -2122,7 +2122,7 @@
       </c>
     </row>
     <row r="7" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="37"/>
+      <c r="A7" s="42"/>
       <c r="B7" s="8" t="s">
         <v>6</v>
       </c>
@@ -2380,7 +2380,7 @@
       </c>
     </row>
     <row r="8" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="37"/>
+      <c r="A8" s="42"/>
       <c r="B8" s="8" t="s">
         <v>7</v>
       </c>
@@ -2638,7 +2638,7 @@
       </c>
     </row>
     <row r="9" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="37"/>
+      <c r="A9" s="42"/>
       <c r="B9" s="8" t="s">
         <v>8</v>
       </c>
@@ -2896,7 +2896,7 @@
       </c>
     </row>
     <row r="10" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="37"/>
+      <c r="A10" s="42"/>
       <c r="B10" s="8" t="s">
         <v>9</v>
       </c>
@@ -3154,7 +3154,7 @@
       </c>
     </row>
     <row r="11" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="37"/>
+      <c r="A11" s="42"/>
       <c r="B11" s="8" t="s">
         <v>10</v>
       </c>
@@ -3412,7 +3412,7 @@
       </c>
     </row>
     <row r="12" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="37"/>
+      <c r="A12" s="42"/>
       <c r="B12" s="8" t="s">
         <v>11</v>
       </c>
@@ -3670,7 +3670,7 @@
       </c>
     </row>
     <row r="13" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="37"/>
+      <c r="A13" s="42"/>
       <c r="B13" s="8" t="s">
         <v>12</v>
       </c>
@@ -3928,7 +3928,7 @@
       </c>
     </row>
     <row r="14" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="37"/>
+      <c r="A14" s="42"/>
       <c r="B14" s="8" t="s">
         <v>13</v>
       </c>
@@ -4186,7 +4186,7 @@
       </c>
     </row>
     <row r="15" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="37"/>
+      <c r="A15" s="42"/>
       <c r="B15" s="8" t="s">
         <v>14</v>
       </c>
@@ -4444,7 +4444,7 @@
       </c>
     </row>
     <row r="16" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="37"/>
+      <c r="A16" s="42"/>
       <c r="B16" s="8" t="s">
         <v>15</v>
       </c>
@@ -4702,7 +4702,7 @@
       </c>
     </row>
     <row r="17" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="37"/>
+      <c r="A17" s="42"/>
       <c r="B17" s="8" t="s">
         <v>16</v>
       </c>
@@ -4960,7 +4960,7 @@
       </c>
     </row>
     <row r="18" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="37"/>
+      <c r="A18" s="42"/>
       <c r="B18" s="8" t="s">
         <v>17</v>
       </c>
@@ -5218,7 +5218,7 @@
       </c>
     </row>
     <row r="19" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="37"/>
+      <c r="A19" s="42"/>
       <c r="B19" s="8" t="s">
         <v>18</v>
       </c>
@@ -5476,7 +5476,7 @@
       </c>
     </row>
     <row r="20" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="37"/>
+      <c r="A20" s="42"/>
       <c r="B20" s="8" t="s">
         <v>19</v>
       </c>
@@ -5734,7 +5734,7 @@
       </c>
     </row>
     <row r="21" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="37"/>
+      <c r="A21" s="42"/>
       <c r="B21" s="8" t="s">
         <v>20</v>
       </c>
@@ -5992,7 +5992,7 @@
       </c>
     </row>
     <row r="22" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="37"/>
+      <c r="A22" s="42"/>
       <c r="B22" s="8" t="s">
         <v>21</v>
       </c>
@@ -6250,7 +6250,7 @@
       </c>
     </row>
     <row r="23" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="37"/>
+      <c r="A23" s="42"/>
       <c r="B23" s="8" t="s">
         <v>22</v>
       </c>
@@ -6508,7 +6508,7 @@
       </c>
     </row>
     <row r="24" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="37"/>
+      <c r="A24" s="42"/>
       <c r="B24" s="8" t="s">
         <v>23</v>
       </c>
@@ -6766,7 +6766,7 @@
       </c>
     </row>
     <row r="25" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="37"/>
+      <c r="A25" s="42"/>
       <c r="B25" s="8" t="s">
         <v>24</v>
       </c>
@@ -7024,7 +7024,7 @@
       </c>
     </row>
     <row r="26" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="37"/>
+      <c r="A26" s="42"/>
       <c r="B26" s="8" t="s">
         <v>25</v>
       </c>
@@ -7282,7 +7282,7 @@
       </c>
     </row>
     <row r="27" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="37"/>
+      <c r="A27" s="42"/>
       <c r="B27" s="8" t="s">
         <v>26</v>
       </c>
@@ -7540,7 +7540,7 @@
       </c>
     </row>
     <row r="28" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="37"/>
+      <c r="A28" s="42"/>
       <c r="B28" s="8" t="s">
         <v>27</v>
       </c>
@@ -7798,7 +7798,7 @@
       </c>
     </row>
     <row r="29" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="37"/>
+      <c r="A29" s="42"/>
       <c r="B29" s="8" t="s">
         <v>28</v>
       </c>
@@ -8056,7 +8056,7 @@
       </c>
     </row>
     <row r="30" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="37"/>
+      <c r="A30" s="42"/>
       <c r="B30" s="8" t="s">
         <v>29</v>
       </c>
@@ -8314,7 +8314,7 @@
       </c>
     </row>
     <row r="31" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="37"/>
+      <c r="A31" s="42"/>
       <c r="B31" s="8" t="s">
         <v>30</v>
       </c>
@@ -8572,7 +8572,7 @@
       </c>
     </row>
     <row r="32" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="37"/>
+      <c r="A32" s="42"/>
       <c r="B32" s="8" t="s">
         <v>31</v>
       </c>
@@ -8830,7 +8830,7 @@
       </c>
     </row>
     <row r="33" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="37"/>
+      <c r="A33" s="42"/>
       <c r="B33" s="8" t="s">
         <v>32</v>
       </c>
@@ -9088,7 +9088,7 @@
       </c>
     </row>
     <row r="34" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="37"/>
+      <c r="A34" s="42"/>
       <c r="B34" s="8" t="s">
         <v>33</v>
       </c>
@@ -9346,7 +9346,7 @@
       </c>
     </row>
     <row r="35" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="37"/>
+      <c r="A35" s="42"/>
       <c r="B35" s="8" t="s">
         <v>34</v>
       </c>
@@ -9582,7 +9582,7 @@
       </c>
     </row>
     <row r="36" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="38"/>
+      <c r="A36" s="43"/>
       <c r="B36" s="8" t="s">
         <v>35</v>
       </c>
@@ -9840,7 +9840,7 @@
       </c>
     </row>
     <row r="37" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="45" t="s">
+      <c r="A37" s="50" t="s">
         <v>36</v>
       </c>
       <c r="B37" s="9" t="s">
@@ -10100,7 +10100,7 @@
       </c>
     </row>
     <row r="38" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="46"/>
+      <c r="A38" s="51"/>
       <c r="B38" s="9" t="s">
         <v>38</v>
       </c>
@@ -10358,7 +10358,7 @@
       </c>
     </row>
     <row r="39" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="46"/>
+      <c r="A39" s="51"/>
       <c r="B39" s="9" t="s">
         <v>39</v>
       </c>
@@ -10616,7 +10616,7 @@
       </c>
     </row>
     <row r="40" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="46"/>
+      <c r="A40" s="51"/>
       <c r="B40" s="9" t="s">
         <v>40</v>
       </c>
@@ -10874,7 +10874,7 @@
       </c>
     </row>
     <row r="41" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="46"/>
+      <c r="A41" s="51"/>
       <c r="B41" s="9" t="s">
         <v>41</v>
       </c>
@@ -11132,7 +11132,7 @@
       </c>
     </row>
     <row r="42" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A42" s="46"/>
+      <c r="A42" s="51"/>
       <c r="B42" s="9" t="s">
         <v>42</v>
       </c>
@@ -11390,7 +11390,7 @@
       </c>
     </row>
     <row r="43" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A43" s="46"/>
+      <c r="A43" s="51"/>
       <c r="B43" s="9" t="s">
         <v>43</v>
       </c>
@@ -11648,7 +11648,7 @@
       </c>
     </row>
     <row r="44" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A44" s="46"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="9" t="s">
         <v>87</v>
       </c>
@@ -11906,7 +11906,7 @@
       </c>
     </row>
     <row r="45" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A45" s="46"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="9" t="s">
         <v>44</v>
       </c>
@@ -12164,7 +12164,7 @@
       </c>
     </row>
     <row r="46" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A46" s="47"/>
+      <c r="A46" s="52"/>
       <c r="B46" s="9" t="s">
         <v>92</v>
       </c>
@@ -12422,7 +12422,7 @@
       </c>
     </row>
     <row r="47" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="39" t="s">
+      <c r="A47" s="44" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="10" t="s">
@@ -12682,7 +12682,7 @@
       </c>
     </row>
     <row r="48" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A48" s="40"/>
+      <c r="A48" s="45"/>
       <c r="B48" s="10" t="s">
         <v>46</v>
       </c>
@@ -12940,7 +12940,7 @@
       </c>
     </row>
     <row r="49" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A49" s="40"/>
+      <c r="A49" s="45"/>
       <c r="B49" s="10" t="s">
         <v>47</v>
       </c>
@@ -13198,7 +13198,7 @@
       </c>
     </row>
     <row r="50" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A50" s="40"/>
+      <c r="A50" s="45"/>
       <c r="B50" s="10" t="s">
         <v>48</v>
       </c>
@@ -13456,7 +13456,7 @@
       </c>
     </row>
     <row r="51" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A51" s="40"/>
+      <c r="A51" s="45"/>
       <c r="B51" s="10" t="s">
         <v>49</v>
       </c>
@@ -13714,7 +13714,7 @@
       </c>
     </row>
     <row r="52" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A52" s="41"/>
+      <c r="A52" s="46"/>
       <c r="B52" s="10" t="s">
         <v>50</v>
       </c>
@@ -13972,7 +13972,7 @@
       </c>
     </row>
     <row r="53" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="42" t="s">
+      <c r="A53" s="47" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="11" t="s">
@@ -14232,7 +14232,7 @@
       </c>
     </row>
     <row r="54" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="43"/>
+      <c r="A54" s="48"/>
       <c r="B54" s="11" t="s">
         <v>53</v>
       </c>
@@ -14490,7 +14490,7 @@
       </c>
     </row>
     <row r="55" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A55" s="44"/>
+      <c r="A55" s="49"/>
       <c r="B55" s="11" t="s">
         <v>93</v>
       </c>
@@ -14586,7 +14586,7 @@
       <c r="CH55" s="20"/>
     </row>
     <row r="56" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A56" s="53" t="s">
+      <c r="A56" s="58" t="s">
         <v>54</v>
       </c>
       <c r="B56" s="12" t="s">
@@ -14846,7 +14846,7 @@
       </c>
     </row>
     <row r="57" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A57" s="54"/>
+      <c r="A57" s="59"/>
       <c r="B57" s="12" t="s">
         <v>56</v>
       </c>
@@ -15094,7 +15094,7 @@
       </c>
     </row>
     <row r="58" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A58" s="54"/>
+      <c r="A58" s="59"/>
       <c r="B58" s="12" t="s">
         <v>57</v>
       </c>
@@ -15352,7 +15352,7 @@
       </c>
     </row>
     <row r="59" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A59" s="54"/>
+      <c r="A59" s="59"/>
       <c r="B59" s="12" t="s">
         <v>58</v>
       </c>
@@ -15610,7 +15610,7 @@
       </c>
     </row>
     <row r="60" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A60" s="54"/>
+      <c r="A60" s="59"/>
       <c r="B60" s="12" t="s">
         <v>59</v>
       </c>
@@ -15868,7 +15868,7 @@
       </c>
     </row>
     <row r="61" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A61" s="55"/>
+      <c r="A61" s="60"/>
       <c r="B61" s="12" t="s">
         <v>60</v>
       </c>
@@ -16126,7 +16126,7 @@
       </c>
     </row>
     <row r="62" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A62" s="56" t="s">
+      <c r="A62" s="61" t="s">
         <v>61</v>
       </c>
       <c r="B62" s="13" t="s">
@@ -16386,7 +16386,7 @@
       </c>
     </row>
     <row r="63" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A63" s="57"/>
+      <c r="A63" s="62"/>
       <c r="B63" s="13" t="s">
         <v>85</v>
       </c>
@@ -16644,7 +16644,7 @@
       </c>
     </row>
     <row r="64" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A64" s="50" t="s">
+      <c r="A64" s="55" t="s">
         <v>63</v>
       </c>
       <c r="B64" s="14" t="s">
@@ -16888,7 +16888,7 @@
         <v>95519.230769230766</v>
       </c>
       <c r="CD64" s="23">
-        <v>71821.084615384621</v>
+        <v>99213.846153846156</v>
       </c>
       <c r="CE64" s="23">
         <v>0</v>
@@ -16904,7 +16904,7 @@
       </c>
     </row>
     <row r="65" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A65" s="51"/>
+      <c r="A65" s="56"/>
       <c r="B65" s="14" t="s">
         <v>65</v>
       </c>
@@ -17146,7 +17146,7 @@
         <v>95461.538461538454</v>
       </c>
       <c r="CD65" s="23">
-        <v>84073.992307692301</v>
+        <v>108016.92307692308</v>
       </c>
       <c r="CE65" s="23">
         <v>0</v>
@@ -17162,7 +17162,7 @@
       </c>
     </row>
     <row r="66" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" s="51"/>
+      <c r="A66" s="56"/>
       <c r="B66" s="14" t="s">
         <v>66</v>
       </c>
@@ -17420,7 +17420,7 @@
       </c>
     </row>
     <row r="67" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" s="52"/>
+      <c r="A67" s="57"/>
       <c r="B67" s="14" t="s">
         <v>84</v>
       </c>
@@ -17662,7 +17662,7 @@
         <v>55020.869230769233</v>
       </c>
       <c r="CD67" s="23">
-        <v>35205.461538461539</v>
+        <v>48487.769230769227</v>
       </c>
       <c r="CE67" s="23">
         <v>0</v>
@@ -17678,7 +17678,7 @@
       </c>
     </row>
     <row r="68" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A68" s="58" t="s">
+      <c r="A68" s="63" t="s">
         <v>67</v>
       </c>
       <c r="B68" s="15" t="s">
@@ -17938,7 +17938,7 @@
       </c>
     </row>
     <row r="69" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A69" s="59"/>
+      <c r="A69" s="64"/>
       <c r="B69" s="15" t="s">
         <v>69</v>
       </c>
@@ -18196,7 +18196,7 @@
       </c>
     </row>
     <row r="70" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A70" s="60"/>
+      <c r="A70" s="65"/>
       <c r="B70" s="15" t="s">
         <v>70</v>
       </c>
@@ -18974,7 +18974,7 @@
       </c>
     </row>
     <row r="73" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A73" s="42" t="s">
+      <c r="A73" s="47" t="s">
         <v>75</v>
       </c>
       <c r="B73" s="11" t="s">
@@ -19234,7 +19234,7 @@
       </c>
     </row>
     <row r="74" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A74" s="43"/>
+      <c r="A74" s="48"/>
       <c r="B74" s="11" t="s">
         <v>77</v>
       </c>
@@ -19492,7 +19492,7 @@
       </c>
     </row>
     <row r="75" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A75" s="43"/>
+      <c r="A75" s="48"/>
       <c r="B75" s="11" t="s">
         <v>78</v>
       </c>
@@ -19750,7 +19750,7 @@
       </c>
     </row>
     <row r="76" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A76" s="43"/>
+      <c r="A76" s="48"/>
       <c r="B76" s="11" t="s">
         <v>79</v>
       </c>
@@ -20008,7 +20008,7 @@
       </c>
     </row>
     <row r="77" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A77" s="44"/>
+      <c r="A77" s="49"/>
       <c r="B77" s="11" t="s">
         <v>80</v>
       </c>
@@ -20266,7 +20266,7 @@
       </c>
     </row>
     <row r="78" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A78" s="48" t="s">
+      <c r="A78" s="53" t="s">
         <v>81</v>
       </c>
       <c r="B78" s="5" t="s">
@@ -20526,7 +20526,7 @@
       </c>
     </row>
     <row r="79" spans="1:86" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" s="49"/>
+      <c r="A79" s="54"/>
       <c r="B79" s="5" t="s">
         <v>83</v>
       </c>
@@ -20785,15 +20785,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="AY3:BJ3"/>
-    <mergeCell ref="C2:CH2"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="BK3:BV3"/>
-    <mergeCell ref="BW3:CH3"/>
-    <mergeCell ref="C3:N3"/>
-    <mergeCell ref="O3:Z3"/>
-    <mergeCell ref="AA3:AL3"/>
-    <mergeCell ref="AM3:AX3"/>
     <mergeCell ref="A5:A36"/>
     <mergeCell ref="A47:A52"/>
     <mergeCell ref="A53:A55"/>
@@ -20804,6 +20795,15 @@
     <mergeCell ref="A56:A61"/>
     <mergeCell ref="A62:A63"/>
     <mergeCell ref="A68:A70"/>
+    <mergeCell ref="AY3:BJ3"/>
+    <mergeCell ref="C2:CH2"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="BK3:BV3"/>
+    <mergeCell ref="BW3:CH3"/>
+    <mergeCell ref="C3:N3"/>
+    <mergeCell ref="O3:Z3"/>
+    <mergeCell ref="AA3:AL3"/>
+    <mergeCell ref="AM3:AX3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="28" orientation="landscape" r:id="rId1"/>

</xml_diff>